<commit_message>
Normalize Feray Fildişi in October schedule
</commit_message>
<xml_diff>
--- a/ekim2026.xlsx
+++ b/ekim2026.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa1" sheetId="1" r:id="Rad6f53dec3404229"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa1" sheetId="1" r:id="R165485f64c3f4762"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,9 +350,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">ALİ SERHAT AKSU </x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FERAY FİLDİĞİ</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">BEŞİR ARMANÇ GÜMÜŞÇÜ</x:t>
@@ -2275,8 +2272,8 @@
       <x:c r="M28" s="5" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="N28" s="5" t="s">
-        <x:v>114</x:v>
+      <x:c r="N28" s="5" t="str">
+        <x:v>FERAY FİLDİŞİ</x:v>
       </x:c>
       <x:c r="O28" s="5" t="s">
         <x:v>85</x:v>
@@ -2339,7 +2336,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="P29" s="5" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="Q29" s="5"/>
       <x:c r="R29" s="5"/>
@@ -2453,7 +2450,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="P31" s="5" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="Q31" s="5"/>
       <x:c r="R31" s="5"/>

</xml_diff>